<commit_message>
Finalize Smartup A2 flows, form timeouts, and navigation validation
</commit_message>
<xml_diff>
--- a/outputs/a2-migration-01a0e663/a2-internal-tracker.xlsx
+++ b/outputs/a2-migration-01a0e663/a2-internal-tracker.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Holat" sheetId="1" r:id="Rc1d9557526244c8a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Formalar" sheetId="2" r:id="Re281485fe0d74132"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Testcaselar" sheetId="3" r:id="R4c0ad884f4154461"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Runlar" sheetId="4" r:id="Ra1370fed6e01477a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Muammolar" sheetId="5" r:id="R57218ee9b1d8443e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nashr tarixi" sheetId="6" r:id="R365ea4ac034646b7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Holat" sheetId="1" r:id="Rdde95688102b402a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Formalar" sheetId="2" r:id="R586477ae46fe4993"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Testcaselar" sheetId="3" r:id="R45ecc8504ae2475c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Runlar" sheetId="4" r:id="Rd1106f312ef3455b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Muammolar" sheetId="5" r:id="R19ac250de9f94073"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nashr tarixi" sheetId="6" r:id="Rbbd31a89c11643bf"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -86,7 +86,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="20">
+  <x:cellXfs count="25">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -129,6 +129,21 @@
     <x:xf numFmtId="201" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="200" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -136,77 +151,77 @@
   <x:dxfs count="11">
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDE9E7"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF1CC"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF1CC"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF1CC"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDE9E7"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDE9E7"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF1CC"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF1CC"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF1CC"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDE9E7"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDE9E7"/>
         </x:patternFill>
       </x:fill>
@@ -243,7 +258,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="CasesTable" displayName="CasesTable" ref="A5:K6" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="CasesTable" displayName="CasesTable" ref="A5:K27" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="Case ID"/>
     <x:tableColumn id="2" name="Forma ID"/>
@@ -262,7 +277,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="RunsTable" displayName="RunsTable" ref="A5:N6" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="RunsTable" displayName="RunsTable" ref="A5:N29" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="14">
     <x:tableColumn id="1" name="Run ID"/>
     <x:tableColumn id="2" name="Case ID"/>
@@ -601,7 +616,7 @@
       </x:c>
       <x:c r="B6" s="17" t="n">
         <x:f>COUNTIFS('Formalar'!G6:G5005,"not_tested")</x:f>
-        <x:v>1009</x:v>
+        <x:v>1003</x:v>
       </x:c>
       <x:c r="C6" s="1"/>
       <x:c r="D6" s="1"/>
@@ -648,7 +663,7 @@
       </x:c>
       <x:c r="B9" s="17" t="n">
         <x:f>COUNTIFS('Formalar'!G6:G5005,"failed")</x:f>
-        <x:v>0</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="C9" s="1"/>
       <x:c r="D9" s="1" t="str">
@@ -680,7 +695,7 @@
       </x:c>
       <x:c r="B11" s="17" t="n">
         <x:f>COUNTIFS('Formalar'!G6:G5005,"needs_review")</x:f>
-        <x:v>0</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="C11" s="1"/>
       <x:c r="D11" s="1" t="str">
@@ -697,7 +712,7 @@
       </x:c>
       <x:c r="B12" s="17" t="n">
         <x:f>COUNTA('Testcaselar'!A6:A5005)</x:f>
-        <x:v>0</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="C12" s="1"/>
       <x:c r="D12" s="1"/>
@@ -712,11 +727,11 @@
       </x:c>
       <x:c r="B13" s="17" t="n">
         <x:f>COUNTA('Runlar'!A6:A5005)</x:f>
-        <x:v>0</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="C13" s="1"/>
       <x:c r="D13" s="1" t="str">
-        <x:v>0 muammo: hozircha tekshiruv bajarilmagan.</x:v>
+        <x:v>Supplier pilot: SUP-001 ochiq; nashr qilinmagan.</x:v>
       </x:c>
       <x:c r="E13" s="1"/>
       <x:c r="F13" s="1"/>
@@ -729,7 +744,7 @@
       </x:c>
       <x:c r="B14" s="17" t="n">
         <x:f>COUNTA('Muammolar'!A6:A5005)</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="C14" s="1"/>
       <x:c r="D14" s="1"/>
@@ -7813,19 +7828,29 @@
         <x:v>/anor/mkw/supplier_list</x:v>
       </x:c>
       <x:c r="G163" s="10" t="str">
-        <x:v>not_tested</x:v>
-      </x:c>
-      <x:c r="H163" s="10" t="str"/>
-      <x:c r="I163" s="10" t="str"/>
-      <x:c r="J163" s="10" t="str"/>
+        <x:v>needs_review</x:v>
+      </x:c>
+      <x:c r="H163" s="10" t="str">
+        <x:v>add: pilot qamrovi; supplier-20260928.md</x:v>
+      </x:c>
+      <x:c r="I163" s="10" t="str">
+        <x:v>Xtrade A2 / Admin / filial-pw157168</x:v>
+      </x:c>
+      <x:c r="J163" s="10" t="str">
+        <x:v>SUP-R03</x:v>
+      </x:c>
       <x:c r="K163" s="10" t="str"/>
-      <x:c r="L163" s="10" t="str"/>
-      <x:c r="M163" s="10" t="str"/>
+      <x:c r="L163" s="10" t="str">
+        <x:v>skills/smartup-guide/references/forms/supplier.md</x:v>
+      </x:c>
+      <x:c r="M163" s="10" t="str">
+        <x:v>tests/smoke/test_suppliers/test_01_supplier_purchase_tab.py::test_supplier_purchase_tab</x:v>
+      </x:c>
       <x:c r="N163" s="10" t="str">
-        <x:v>not_planned</x:v>
+        <x:v>written_not_run</x:v>
       </x:c>
       <x:c r="O163" s="10" t="str">
-        <x:v>pending</x:v>
+        <x:v>needs_review</x:v>
       </x:c>
       <x:c r="P163" s="10" t="str">
         <x:v>not_published</x:v>
@@ -7856,19 +7881,31 @@
         <x:v>/anor/mkw/supplier_list</x:v>
       </x:c>
       <x:c r="G164" s="10" t="str">
-        <x:v>not_tested</x:v>
-      </x:c>
-      <x:c r="H164" s="10" t="str"/>
-      <x:c r="I164" s="10" t="str"/>
-      <x:c r="J164" s="10" t="str"/>
-      <x:c r="K164" s="10" t="str"/>
-      <x:c r="L164" s="10" t="str"/>
-      <x:c r="M164" s="10" t="str"/>
+        <x:v>failed</x:v>
+      </x:c>
+      <x:c r="H164" s="10" t="str">
+        <x:v>Logical supplier CRUD + single/multiple + search/filter; SUP-001 open</x:v>
+      </x:c>
+      <x:c r="I164" s="10" t="str">
+        <x:v>Xtrade A2 / Admin / filial-pw157168</x:v>
+      </x:c>
+      <x:c r="J164" s="10" t="str">
+        <x:v>SUP-R22</x:v>
+      </x:c>
+      <x:c r="K164" s="10" t="str">
+        <x:v>SUP-001</x:v>
+      </x:c>
+      <x:c r="L164" s="10" t="str">
+        <x:v>skills/smartup-guide/references/forms/supplier.md</x:v>
+      </x:c>
+      <x:c r="M164" s="10" t="str">
+        <x:v>tests/smoke/test_suppliers/test_01_supplier_purchase_tab.py::test_supplier_purchase_tab</x:v>
+      </x:c>
       <x:c r="N164" s="10" t="str">
-        <x:v>not_planned</x:v>
+        <x:v>written_not_run</x:v>
       </x:c>
       <x:c r="O164" s="10" t="str">
-        <x:v>pending</x:v>
+        <x:v>needs_review</x:v>
       </x:c>
       <x:c r="P164" s="10" t="str">
         <x:v>not_published</x:v>
@@ -7899,19 +7936,27 @@
         <x:v>/anor/mkw/supplier_list</x:v>
       </x:c>
       <x:c r="G165" s="10" t="str">
-        <x:v>not_tested</x:v>
-      </x:c>
-      <x:c r="H165" s="10" t="str"/>
-      <x:c r="I165" s="10" t="str"/>
-      <x:c r="J165" s="10" t="str"/>
+        <x:v>needs_review</x:v>
+      </x:c>
+      <x:c r="H165" s="10" t="str">
+        <x:v>product: pilot qamrovi; supplier-20260928.md</x:v>
+      </x:c>
+      <x:c r="I165" s="10" t="str">
+        <x:v>Xtrade A2 / Admin / filial-pw157168</x:v>
+      </x:c>
+      <x:c r="J165" s="10" t="str">
+        <x:v>SUP-R12</x:v>
+      </x:c>
       <x:c r="K165" s="10" t="str"/>
-      <x:c r="L165" s="10" t="str"/>
+      <x:c r="L165" s="10" t="str">
+        <x:v>skills/smartup-guide/references/forms/supplier.md</x:v>
+      </x:c>
       <x:c r="M165" s="10" t="str"/>
       <x:c r="N165" s="10" t="str">
         <x:v>not_planned</x:v>
       </x:c>
       <x:c r="O165" s="10" t="str">
-        <x:v>pending</x:v>
+        <x:v>needs_review</x:v>
       </x:c>
       <x:c r="P165" s="10" t="str">
         <x:v>not_published</x:v>
@@ -40020,19 +40065,27 @@
         <x:v>/anor/mkw/input/file_list</x:v>
       </x:c>
       <x:c r="G912" s="10" t="str">
-        <x:v>not_tested</x:v>
-      </x:c>
-      <x:c r="H912" s="10" t="str"/>
-      <x:c r="I912" s="10" t="str"/>
-      <x:c r="J912" s="10" t="str"/>
+        <x:v>needs_review</x:v>
+      </x:c>
+      <x:c r="H912" s="10" t="str">
+        <x:v>audit: pilot qamrovi; supplier-20260928.md</x:v>
+      </x:c>
+      <x:c r="I912" s="10" t="str">
+        <x:v>Xtrade A2 / Admin / filial-pw157168</x:v>
+      </x:c>
+      <x:c r="J912" s="10" t="str">
+        <x:v>SUP-R19</x:v>
+      </x:c>
       <x:c r="K912" s="10" t="str"/>
-      <x:c r="L912" s="10" t="str"/>
+      <x:c r="L912" s="10" t="str">
+        <x:v>skills/smartup-guide/references/forms/supplier.md</x:v>
+      </x:c>
       <x:c r="M912" s="10" t="str"/>
       <x:c r="N912" s="10" t="str">
         <x:v>not_planned</x:v>
       </x:c>
       <x:c r="O912" s="10" t="str">
-        <x:v>pending</x:v>
+        <x:v>needs_review</x:v>
       </x:c>
       <x:c r="P912" s="10" t="str">
         <x:v>not_published</x:v>
@@ -40192,19 +40245,27 @@
         <x:v>/anor/mkw/input/file_list</x:v>
       </x:c>
       <x:c r="G916" s="10" t="str">
-        <x:v>not_tested</x:v>
-      </x:c>
-      <x:c r="H916" s="10" t="str"/>
-      <x:c r="I916" s="10" t="str"/>
-      <x:c r="J916" s="10" t="str"/>
+        <x:v>needs_review</x:v>
+      </x:c>
+      <x:c r="H916" s="10" t="str">
+        <x:v>edit: pilot qamrovi; supplier-20260928.md</x:v>
+      </x:c>
+      <x:c r="I916" s="10" t="str">
+        <x:v>Xtrade A2 / Admin / filial-pw157168</x:v>
+      </x:c>
+      <x:c r="J916" s="10" t="str">
+        <x:v>SUP-R07</x:v>
+      </x:c>
       <x:c r="K916" s="10" t="str"/>
-      <x:c r="L916" s="10" t="str"/>
+      <x:c r="L916" s="10" t="str">
+        <x:v>skills/smartup-guide/references/forms/supplier.md</x:v>
+      </x:c>
       <x:c r="M916" s="10" t="str"/>
       <x:c r="N916" s="10" t="str">
         <x:v>not_planned</x:v>
       </x:c>
       <x:c r="O916" s="10" t="str">
-        <x:v>pending</x:v>
+        <x:v>needs_review</x:v>
       </x:c>
       <x:c r="P916" s="10" t="str">
         <x:v>not_published</x:v>
@@ -40450,19 +40511,31 @@
         <x:v>/anor/mkw/input/file_list</x:v>
       </x:c>
       <x:c r="G922" s="10" t="str">
-        <x:v>not_tested</x:v>
-      </x:c>
-      <x:c r="H922" s="10" t="str"/>
-      <x:c r="I922" s="10" t="str"/>
-      <x:c r="J922" s="10" t="str"/>
-      <x:c r="K922" s="10" t="str"/>
-      <x:c r="L922" s="10" t="str"/>
-      <x:c r="M922" s="10" t="str"/>
+        <x:v>failed</x:v>
+      </x:c>
+      <x:c r="H922" s="10" t="str">
+        <x:v>view: pilot qamrovi; supplier-20260928.md</x:v>
+      </x:c>
+      <x:c r="I922" s="10" t="str">
+        <x:v>Xtrade A2 / Admin / filial-pw157168</x:v>
+      </x:c>
+      <x:c r="J922" s="10" t="str">
+        <x:v>SUP-R06b</x:v>
+      </x:c>
+      <x:c r="K922" s="10" t="str">
+        <x:v>SUP-001</x:v>
+      </x:c>
+      <x:c r="L922" s="10" t="str">
+        <x:v>skills/smartup-guide/references/forms/supplier.md</x:v>
+      </x:c>
+      <x:c r="M922" s="10" t="str">
+        <x:v>tests/smoke/test_suppliers/test_01_supplier_purchase_tab.py::test_supplier_purchase_tab</x:v>
+      </x:c>
       <x:c r="N922" s="10" t="str">
-        <x:v>not_planned</x:v>
+        <x:v>written_not_run</x:v>
       </x:c>
       <x:c r="O922" s="10" t="str">
-        <x:v>pending</x:v>
+        <x:v>needs_review</x:v>
       </x:c>
       <x:c r="P922" s="10" t="str">
         <x:v>not_published</x:v>
@@ -44467,7 +44540,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4d0bc8b8a67b4d40"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R43697bcd402a46d7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -44519,7 +44592,7 @@
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
       <x:c r="A3" s="4" t="str">
-        <x:v>Hozircha testcase yozilmagan. Reja va bajarilgan natija Runlar orqali ajratiladi.</x:v>
+        <x:v>22 testcase; amaldagi natija va urinishlar Runlar varag‘ida.</x:v>
       </x:c>
       <x:c r="B3" s="2"/>
       <x:c r="C3" s="2"/>
@@ -44580,18 +44653,733 @@
         <x:v>Manba / dalil</x:v>
       </x:c>
     </x:row>
-    <x:row r="6" ht="24" customHeight="1">
-      <x:c r="A6" s="2"/>
-      <x:c r="B6" s="2"/>
-      <x:c r="C6" s="2"/>
-      <x:c r="D6" s="2"/>
-      <x:c r="E6" s="2"/>
-      <x:c r="F6" s="2"/>
-      <x:c r="G6" s="2"/>
-      <x:c r="H6" s="2"/>
-      <x:c r="I6" s="2"/>
-      <x:c r="J6" s="2"/>
-      <x:c r="K6" s="2"/>
+    <x:row r="6" ht="72" customHeight="1">
+      <x:c r="A6" s="9" t="str">
+        <x:v>SUP-01</x:v>
+      </x:c>
+      <x:c r="B6" s="9" t="str">
+        <x:v>A2-c6398bcf3bba</x:v>
+      </x:c>
+      <x:c r="C6" s="9" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D6" s="9" t="str">
+        <x:v>Add maydon inventari</x:v>
+      </x:c>
+      <x:c r="E6" s="9" t="str">
+        <x:v>Own A/B/C supplier fixtures; reportdagi data aliaslar</x:v>
+      </x:c>
+      <x:c r="F6" s="9" t="str">
+        <x:v>Bo‘sh addni ochish; required holat va switchlarni aniqlash</x:v>
+      </x:c>
+      <x:c r="G6" s="9" t="str">
+        <x:v>Name bo‘shligida Save disabled; VAT yoqilganda percent input</x:v>
+      </x:c>
+      <x:c r="H6" s="9" t="str">
+        <x:v>functional</x:v>
+      </x:c>
+      <x:c r="I6" s="9" t="str">
+        <x:v>ready</x:v>
+      </x:c>
+      <x:c r="J6" s="9" t="str"/>
+      <x:c r="K6" s="9" t="str">
+        <x:v>outputs/a2-migration-01a0e663/supplier-20260928.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="72" customHeight="1">
+      <x:c r="A7" s="9" t="str">
+        <x:v>SUP-02</x:v>
+      </x:c>
+      <x:c r="B7" s="9" t="str">
+        <x:v>A2-c6398bcf3bba</x:v>
+      </x:c>
+      <x:c r="C7" s="9" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D7" s="9" t="str">
+        <x:v>Legal supplier create/save/list</x:v>
+      </x:c>
+      <x:c r="E7" s="9" t="str">
+        <x:v>Own A/B/C supplier fixtures; reportdagi data aliaslar</x:v>
+      </x:c>
+      <x:c r="F7" s="9" t="str">
+        <x:v>A VAT12, excise yes; B default; inline shaxs yaratish va supplierni saqlash</x:v>
+      </x:c>
+      <x:c r="G7" s="9" t="str">
+        <x:v>Code/name/type/status listda saqlangan qiymatga mos</x:v>
+      </x:c>
+      <x:c r="H7" s="9" t="str">
+        <x:v>functional</x:v>
+      </x:c>
+      <x:c r="I7" s="9" t="str">
+        <x:v>ready</x:v>
+      </x:c>
+      <x:c r="J7" s="9" t="str"/>
+      <x:c r="K7" s="9" t="str">
+        <x:v>outputs/a2-migration-01a0e663/supplier-20260928.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="72" customHeight="1">
+      <x:c r="A8" s="9" t="str">
+        <x:v>SUP-03</x:v>
+      </x:c>
+      <x:c r="B8" s="9" t="str">
+        <x:v>A2-c6398bcf3bba</x:v>
+      </x:c>
+      <x:c r="C8" s="9" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D8" s="9" t="str">
+        <x:v>Natural supplier create/save/list</x:v>
+      </x:c>
+      <x:c r="E8" s="9" t="str">
+        <x:v>Own A/B/C supplier fixtures; reportdagi data aliaslar</x:v>
+      </x:c>
+      <x:c r="F8" s="9" t="str">
+        <x:v>Type Natural; inline yangi ism va kod; Enter bilan ismni commit; Save; supplier Save</x:v>
+      </x:c>
+      <x:c r="G8" s="9" t="str">
+        <x:v>Natural supplier yaratiladi va listda ko‘rinadi</x:v>
+      </x:c>
+      <x:c r="H8" s="9" t="str">
+        <x:v>functional</x:v>
+      </x:c>
+      <x:c r="I8" s="9" t="str">
+        <x:v>ready</x:v>
+      </x:c>
+      <x:c r="J8" s="9" t="str"/>
+      <x:c r="K8" s="9" t="str">
+        <x:v>outputs/a2-migration-01a0e663/supplier-20260928.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="72" customHeight="1">
+      <x:c r="A9" s="9" t="str">
+        <x:v>SUP-04</x:v>
+      </x:c>
+      <x:c r="B9" s="9" t="str">
+        <x:v>A2-358b793d482a</x:v>
+      </x:c>
+      <x:c r="C9" s="9" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D9" s="9" t="str">
+        <x:v>View qiymatlari</x:v>
+      </x:c>
+      <x:c r="E9" s="9" t="str">
+        <x:v>Own A/B/C supplier fixtures; reportdagi data aliaslar</x:v>
+      </x:c>
+      <x:c r="F9" s="9" t="str">
+        <x:v>A va C row → Просмотреть; code/name/type/status/VATni solishtirish</x:v>
+      </x:c>
+      <x:c r="G9" s="9" t="str">
+        <x:v>View saqlangan qiymatlarni ko‘rsatadi</x:v>
+      </x:c>
+      <x:c r="H9" s="9" t="str">
+        <x:v>functional</x:v>
+      </x:c>
+      <x:c r="I9" s="9" t="str">
+        <x:v>ready</x:v>
+      </x:c>
+      <x:c r="J9" s="9" t="str"/>
+      <x:c r="K9" s="9" t="str">
+        <x:v>outputs/a2-migration-01a0e663/supplier-20260928.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="72" customHeight="1">
+      <x:c r="A10" s="9" t="str">
+        <x:v>SUP-05</x:v>
+      </x:c>
+      <x:c r="B10" s="9" t="str">
+        <x:v>A2-358b793d482a</x:v>
+      </x:c>
+      <x:c r="C10" s="9" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D10" s="9" t="str">
+        <x:v>View boshqa tablari</x:v>
+      </x:c>
+      <x:c r="E10" s="9" t="str">
+        <x:v>Own A/B/C supplier fixtures; reportdagi data aliaslar</x:v>
+      </x:c>
+      <x:c r="F10" s="9" t="str">
+        <x:v>Details/characteristics/files/products/orders/receipts/returns/initial balance/history tablarini ochish</x:v>
+      </x:c>
+      <x:c r="G10" s="9" t="str">
+        <x:v>Tablar xatosiz, fixturega mos bo‘sh yoki history kontenti</x:v>
+      </x:c>
+      <x:c r="H10" s="9" t="str">
+        <x:v>functional</x:v>
+      </x:c>
+      <x:c r="I10" s="9" t="str">
+        <x:v>ready</x:v>
+      </x:c>
+      <x:c r="J10" s="9" t="str"/>
+      <x:c r="K10" s="9" t="str">
+        <x:v>outputs/a2-migration-01a0e663/supplier-20260928.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="72" customHeight="1">
+      <x:c r="A11" s="9" t="str">
+        <x:v>SUP-06</x:v>
+      </x:c>
+      <x:c r="B11" s="9" t="str">
+        <x:v>A2-358b793d482a</x:v>
+      </x:c>
+      <x:c r="C11" s="9" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D11" s="9" t="str">
+        <x:v>Purchase tab</x:v>
+      </x:c>
+      <x:c r="E11" s="9" t="str">
+        <x:v>Own A/B/C supplier fixtures; reportdagi data aliaslar</x:v>
+      </x:c>
+      <x:c r="F11" s="9" t="str">
+        <x:v>Supplier view → Закупки</x:v>
+      </x:c>
+      <x:c r="G11" s="9" t="str">
+        <x:v>Grid yoki empty-state xatosiz ochiladi</x:v>
+      </x:c>
+      <x:c r="H11" s="9" t="str">
+        <x:v>functional</x:v>
+      </x:c>
+      <x:c r="I11" s="9" t="str">
+        <x:v>ready</x:v>
+      </x:c>
+      <x:c r="J11" s="9" t="str">
+        <x:v>tests/smoke/test_suppliers/test_01_supplier_purchase_tab.py::test_supplier_purchase_tab</x:v>
+      </x:c>
+      <x:c r="K11" s="9" t="str">
+        <x:v>outputs/a2-migration-01a0e663/supplier-20260928.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="72" customHeight="1">
+      <x:c r="A12" s="9" t="str">
+        <x:v>SUP-07</x:v>
+      </x:c>
+      <x:c r="B12" s="9" t="str">
+        <x:v>A2-84e0eb5cd0a4</x:v>
+      </x:c>
+      <x:c r="C12" s="9" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D12" s="9" t="str">
+        <x:v>Edit va readback</x:v>
+      </x:c>
+      <x:c r="E12" s="9" t="str">
+        <x:v>Own A/B/C supplier fixtures; reportdagi data aliaslar</x:v>
+      </x:c>
+      <x:c r="F12" s="9" t="str">
+        <x:v>A VAT12→15, excise yes→no, active→inactive; Save; view va editni qayta ochish</x:v>
+      </x:c>
+      <x:c r="G12" s="9" t="str">
+        <x:v>Yangi qiymatlar saqlanadi; type/name o‘zgarmaydi</x:v>
+      </x:c>
+      <x:c r="H12" s="9" t="str">
+        <x:v>functional</x:v>
+      </x:c>
+      <x:c r="I12" s="9" t="str">
+        <x:v>ready</x:v>
+      </x:c>
+      <x:c r="J12" s="9" t="str"/>
+      <x:c r="K12" s="9" t="str">
+        <x:v>outputs/a2-migration-01a0e663/supplier-20260928.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="72" customHeight="1">
+      <x:c r="A13" s="9" t="str">
+        <x:v>SUP-08</x:v>
+      </x:c>
+      <x:c r="B13" s="9" t="str">
+        <x:v>A2-612640976aeb</x:v>
+      </x:c>
+      <x:c r="C13" s="9" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D13" s="9" t="str">
+        <x:v>Single status amallari</x:v>
+      </x:c>
+      <x:c r="E13" s="9" t="str">
+        <x:v>Own A/B/C supplier fixtures; reportdagi data aliaslar</x:v>
+      </x:c>
+      <x:c r="F13" s="9" t="str">
+        <x:v>A inactive→active; C active→inactive; rowni qayta o‘qish</x:v>
+      </x:c>
+      <x:c r="G13" s="9" t="str">
+        <x:v>Faqat tanlangan supplier statusi o‘zgaradi</x:v>
+      </x:c>
+      <x:c r="H13" s="9" t="str">
+        <x:v>functional</x:v>
+      </x:c>
+      <x:c r="I13" s="9" t="str">
+        <x:v>ready</x:v>
+      </x:c>
+      <x:c r="J13" s="9" t="str"/>
+      <x:c r="K13" s="9" t="str">
+        <x:v>outputs/a2-migration-01a0e663/supplier-20260928.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="72" customHeight="1">
+      <x:c r="A14" s="9" t="str">
+        <x:v>SUP-09</x:v>
+      </x:c>
+      <x:c r="B14" s="9" t="str">
+        <x:v>A2-c286a891c1bf</x:v>
+      </x:c>
+      <x:c r="C14" s="9" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D14" s="9" t="str">
+        <x:v>Single attach</x:v>
+      </x:c>
+      <x:c r="E14" s="9" t="str">
+        <x:v>Own A/B/C supplier fixtures; reportdagi data aliaslar</x:v>
+      </x:c>
+      <x:c r="F14" s="9" t="str">
+        <x:v>A → Прикрепить ТМЦ → Available product → Прикрепить → Да</x:v>
+      </x:c>
+      <x:c r="G14" s="9" t="str">
+        <x:v>Product Attached ro‘yxatga o‘tadi</x:v>
+      </x:c>
+      <x:c r="H14" s="9" t="str">
+        <x:v>functional</x:v>
+      </x:c>
+      <x:c r="I14" s="9" t="str">
+        <x:v>ready</x:v>
+      </x:c>
+      <x:c r="J14" s="9" t="str"/>
+      <x:c r="K14" s="9" t="str">
+        <x:v>outputs/a2-migration-01a0e663/supplier-20260928.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="72" customHeight="1">
+      <x:c r="A15" s="9" t="str">
+        <x:v>SUP-10</x:v>
+      </x:c>
+      <x:c r="B15" s="9" t="str">
+        <x:v>A2-c286a891c1bf</x:v>
+      </x:c>
+      <x:c r="C15" s="9" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D15" s="9" t="str">
+        <x:v>Single detach</x:v>
+      </x:c>
+      <x:c r="E15" s="9" t="str">
+        <x:v>Own A/B/C supplier fixtures; reportdagi data aliaslar</x:v>
+      </x:c>
+      <x:c r="F15" s="9" t="str">
+        <x:v>Attached product → Открепить → Да</x:v>
+      </x:c>
+      <x:c r="G15" s="9" t="str">
+        <x:v>Bog‘lanish yo‘qoladi; product Availablega qaytadi</x:v>
+      </x:c>
+      <x:c r="H15" s="9" t="str">
+        <x:v>functional</x:v>
+      </x:c>
+      <x:c r="I15" s="9" t="str">
+        <x:v>ready</x:v>
+      </x:c>
+      <x:c r="J15" s="9" t="str"/>
+      <x:c r="K15" s="9" t="str">
+        <x:v>outputs/a2-migration-01a0e663/supplier-20260928.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="72" customHeight="1">
+      <x:c r="A16" s="9" t="str">
+        <x:v>SUP-11</x:v>
+      </x:c>
+      <x:c r="B16" s="9" t="str">
+        <x:v>A2-c286a891c1bf</x:v>
+      </x:c>
+      <x:c r="C16" s="9" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D16" s="9" t="str">
+        <x:v>Multiple attach</x:v>
+      </x:c>
+      <x:c r="E16" s="9" t="str">
+        <x:v>Own A/B/C supplier fixtures; reportdagi data aliaslar</x:v>
+      </x:c>
+      <x:c r="F16" s="9" t="str">
+        <x:v>Availabledagi 2 productni tanlash → Прикрепить 2 → Да</x:v>
+      </x:c>
+      <x:c r="G16" s="9" t="str">
+        <x:v>Ikkala product Attachedda</x:v>
+      </x:c>
+      <x:c r="H16" s="9" t="str">
+        <x:v>functional</x:v>
+      </x:c>
+      <x:c r="I16" s="9" t="str">
+        <x:v>ready</x:v>
+      </x:c>
+      <x:c r="J16" s="9" t="str"/>
+      <x:c r="K16" s="9" t="str">
+        <x:v>outputs/a2-migration-01a0e663/supplier-20260928.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="72" customHeight="1">
+      <x:c r="A17" s="9" t="str">
+        <x:v>SUP-12</x:v>
+      </x:c>
+      <x:c r="B17" s="9" t="str">
+        <x:v>A2-c286a891c1bf</x:v>
+      </x:c>
+      <x:c r="C17" s="9" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D17" s="9" t="str">
+        <x:v>Multiple detach</x:v>
+      </x:c>
+      <x:c r="E17" s="9" t="str">
+        <x:v>Own A/B/C supplier fixtures; reportdagi data aliaslar</x:v>
+      </x:c>
+      <x:c r="F17" s="9" t="str">
+        <x:v>Attacheddagi 2 product → Открепить 2 → Да</x:v>
+      </x:c>
+      <x:c r="G17" s="9" t="str">
+        <x:v>Ikkala bog‘lanish olib tashlanadi</x:v>
+      </x:c>
+      <x:c r="H17" s="9" t="str">
+        <x:v>functional</x:v>
+      </x:c>
+      <x:c r="I17" s="9" t="str">
+        <x:v>ready</x:v>
+      </x:c>
+      <x:c r="J17" s="9" t="str"/>
+      <x:c r="K17" s="9" t="str">
+        <x:v>outputs/a2-migration-01a0e663/supplier-20260928.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="72" customHeight="1">
+      <x:c r="A18" s="9" t="str">
+        <x:v>SUP-13</x:v>
+      </x:c>
+      <x:c r="B18" s="9" t="str">
+        <x:v>A2-612640976aeb</x:v>
+      </x:c>
+      <x:c r="C18" s="9" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D18" s="9" t="str">
+        <x:v>Name search</x:v>
+      </x:c>
+      <x:c r="E18" s="9" t="str">
+        <x:v>Own A/B/C supplier fixtures; reportdagi data aliaslar</x:v>
+      </x:c>
+      <x:c r="F18" s="9" t="str">
+        <x:v>B nomini qidiruvga kiritish → Enter</x:v>
+      </x:c>
+      <x:c r="G18" s="9" t="str">
+        <x:v>Faqat B qaytadi</x:v>
+      </x:c>
+      <x:c r="H18" s="9" t="str">
+        <x:v>functional</x:v>
+      </x:c>
+      <x:c r="I18" s="9" t="str">
+        <x:v>ready</x:v>
+      </x:c>
+      <x:c r="J18" s="9" t="str"/>
+      <x:c r="K18" s="9" t="str">
+        <x:v>outputs/a2-migration-01a0e663/supplier-20260928.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="72" customHeight="1">
+      <x:c r="A19" s="9" t="str">
+        <x:v>SUP-14</x:v>
+      </x:c>
+      <x:c r="B19" s="9" t="str">
+        <x:v>A2-612640976aeb</x:v>
+      </x:c>
+      <x:c r="C19" s="9" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D19" s="9" t="str">
+        <x:v>Missing search va reset</x:v>
+      </x:c>
+      <x:c r="E19" s="9" t="str">
+        <x:v>Own A/B/C supplier fixtures; reportdagi data aliaslar</x:v>
+      </x:c>
+      <x:c r="F19" s="9" t="str">
+        <x:v>Noyob mavjud bo‘lmagan nom + Enter; klaviatura bilan clear + Enter</x:v>
+      </x:c>
+      <x:c r="G19" s="9" t="str">
+        <x:v>Avval empty, keyin barcha test yozuvlari qaytadi</x:v>
+      </x:c>
+      <x:c r="H19" s="9" t="str">
+        <x:v>functional</x:v>
+      </x:c>
+      <x:c r="I19" s="9" t="str">
+        <x:v>ready</x:v>
+      </x:c>
+      <x:c r="J19" s="9" t="str"/>
+      <x:c r="K19" s="9" t="str">
+        <x:v>outputs/a2-migration-01a0e663/supplier-20260928.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="72" customHeight="1">
+      <x:c r="A20" s="9" t="str">
+        <x:v>SUP-15</x:v>
+      </x:c>
+      <x:c r="B20" s="9" t="str">
+        <x:v>A2-612640976aeb</x:v>
+      </x:c>
+      <x:c r="C20" s="9" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D20" s="9" t="str">
+        <x:v>VAT filter</x:v>
+      </x:c>
+      <x:c r="E20" s="9" t="str">
+        <x:v>Own A/B/C supplier fixtures; reportdagi data aliaslar</x:v>
+      </x:c>
+      <x:c r="F20" s="9" t="str">
+        <x:v>Filter → НДС=Да → Применить</x:v>
+      </x:c>
+      <x:c r="G20" s="9" t="str">
+        <x:v>Faqat VAT yoqilgan A</x:v>
+      </x:c>
+      <x:c r="H20" s="9" t="str">
+        <x:v>functional</x:v>
+      </x:c>
+      <x:c r="I20" s="9" t="str">
+        <x:v>ready</x:v>
+      </x:c>
+      <x:c r="J20" s="9" t="str"/>
+      <x:c r="K20" s="9" t="str">
+        <x:v>outputs/a2-migration-01a0e663/supplier-20260928.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="72" customHeight="1">
+      <x:c r="A21" s="9" t="str">
+        <x:v>SUP-16</x:v>
+      </x:c>
+      <x:c r="B21" s="9" t="str">
+        <x:v>A2-612640976aeb</x:v>
+      </x:c>
+      <x:c r="C21" s="9" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D21" s="9" t="str">
+        <x:v>Status filter va reset</x:v>
+      </x:c>
+      <x:c r="E21" s="9" t="str">
+        <x:v>Own A/B/C supplier fixtures; reportdagi data aliaslar</x:v>
+      </x:c>
+      <x:c r="F21" s="9" t="str">
+        <x:v>A/B inactive paytida Active filter; keyin Показать все</x:v>
+      </x:c>
+      <x:c r="G21" s="9" t="str">
+        <x:v>0/0; resetdan keyin 2/2</x:v>
+      </x:c>
+      <x:c r="H21" s="9" t="str">
+        <x:v>functional</x:v>
+      </x:c>
+      <x:c r="I21" s="9" t="str">
+        <x:v>ready</x:v>
+      </x:c>
+      <x:c r="J21" s="9" t="str"/>
+      <x:c r="K21" s="9" t="str">
+        <x:v>outputs/a2-migration-01a0e663/supplier-20260928.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="72" customHeight="1">
+      <x:c r="A22" s="9" t="str">
+        <x:v>SUP-17</x:v>
+      </x:c>
+      <x:c r="B22" s="9" t="str">
+        <x:v>A2-612640976aeb</x:v>
+      </x:c>
+      <x:c r="C22" s="9" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D22" s="9" t="str">
+        <x:v>Multiple status</x:v>
+      </x:c>
+      <x:c r="E22" s="9" t="str">
+        <x:v>Own A/B/C supplier fixtures; reportdagi data aliaslar</x:v>
+      </x:c>
+      <x:c r="F22" s="9" t="str">
+        <x:v>A/B tanlash; inactive → Да; qayta tanlab active → Да</x:v>
+      </x:c>
+      <x:c r="G22" s="9" t="str">
+        <x:v>Ikkala supplier statuslari mos o‘zgaradi</x:v>
+      </x:c>
+      <x:c r="H22" s="9" t="str">
+        <x:v>functional</x:v>
+      </x:c>
+      <x:c r="I22" s="9" t="str">
+        <x:v>ready</x:v>
+      </x:c>
+      <x:c r="J22" s="9" t="str"/>
+      <x:c r="K22" s="9" t="str">
+        <x:v>outputs/a2-migration-01a0e663/supplier-20260928.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="72" customHeight="1">
+      <x:c r="A23" s="9" t="str">
+        <x:v>SUP-18</x:v>
+      </x:c>
+      <x:c r="B23" s="9" t="str">
+        <x:v>A2-612640976aeb</x:v>
+      </x:c>
+      <x:c r="C23" s="9" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D23" s="9" t="str">
+        <x:v>List history</x:v>
+      </x:c>
+      <x:c r="E23" s="9" t="str">
+        <x:v>Own A/B/C supplier fixtures; reportdagi data aliaslar</x:v>
+      </x:c>
+      <x:c r="F23" s="9" t="str">
+        <x:v>История изменений ochish</x:v>
+      </x:c>
+      <x:c r="G23" s="9" t="str">
+        <x:v>Create/edit/attachment hodisalari mavjud</x:v>
+      </x:c>
+      <x:c r="H23" s="9" t="str">
+        <x:v>functional</x:v>
+      </x:c>
+      <x:c r="I23" s="9" t="str">
+        <x:v>ready</x:v>
+      </x:c>
+      <x:c r="J23" s="9" t="str"/>
+      <x:c r="K23" s="9" t="str">
+        <x:v>outputs/a2-migration-01a0e663/supplier-20260928.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="72" customHeight="1">
+      <x:c r="A24" s="9" t="str">
+        <x:v>SUP-19</x:v>
+      </x:c>
+      <x:c r="B24" s="9" t="str">
+        <x:v>A2-432abf130d2e</x:v>
+      </x:c>
+      <x:c r="C24" s="9" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D24" s="9" t="str">
+        <x:v>Audit details</x:v>
+      </x:c>
+      <x:c r="E24" s="9" t="str">
+        <x:v>Own A/B/C supplier fixtures; reportdagi data aliaslar</x:v>
+      </x:c>
+      <x:c r="F24" s="9" t="str">
+        <x:v>A create hodisasi → Детали</x:v>
+      </x:c>
+      <x:c r="G24" s="9" t="str">
+        <x:v>Supplier A, VAT12/Да, Active</x:v>
+      </x:c>
+      <x:c r="H24" s="9" t="str">
+        <x:v>functional</x:v>
+      </x:c>
+      <x:c r="I24" s="9" t="str">
+        <x:v>ready</x:v>
+      </x:c>
+      <x:c r="J24" s="9" t="str"/>
+      <x:c r="K24" s="9" t="str">
+        <x:v>outputs/a2-migration-01a0e663/supplier-20260928.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="72" customHeight="1">
+      <x:c r="A25" s="9" t="str">
+        <x:v>SUP-20</x:v>
+      </x:c>
+      <x:c r="B25" s="9" t="str">
+        <x:v>A2-612640976aeb</x:v>
+      </x:c>
+      <x:c r="C25" s="9" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D25" s="9" t="str">
+        <x:v>Delete cancel</x:v>
+      </x:c>
+      <x:c r="E25" s="9" t="str">
+        <x:v>Own A/B/C supplier fixtures; reportdagi data aliaslar</x:v>
+      </x:c>
+      <x:c r="F25" s="9" t="str">
+        <x:v>A row → Удалить → Нет</x:v>
+      </x:c>
+      <x:c r="G25" s="9" t="str">
+        <x:v>Supplier saqlanib qoladi</x:v>
+      </x:c>
+      <x:c r="H25" s="9" t="str">
+        <x:v>functional</x:v>
+      </x:c>
+      <x:c r="I25" s="9" t="str">
+        <x:v>ready</x:v>
+      </x:c>
+      <x:c r="J25" s="9" t="str"/>
+      <x:c r="K25" s="9" t="str">
+        <x:v>outputs/a2-migration-01a0e663/supplier-20260928.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="72" customHeight="1">
+      <x:c r="A26" s="9" t="str">
+        <x:v>SUP-21</x:v>
+      </x:c>
+      <x:c r="B26" s="9" t="str">
+        <x:v>A2-612640976aeb</x:v>
+      </x:c>
+      <x:c r="C26" s="9" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D26" s="9" t="str">
+        <x:v>Single delete</x:v>
+      </x:c>
+      <x:c r="E26" s="9" t="str">
+        <x:v>Own A/B/C supplier fixtures; reportdagi data aliaslar</x:v>
+      </x:c>
+      <x:c r="F26" s="9" t="str">
+        <x:v>A row → Удалить → Да; keyinchalik C ham alohida o‘chirish</x:v>
+      </x:c>
+      <x:c r="G26" s="9" t="str">
+        <x:v>Faqat tanlangan test supplier yo‘qoladi</x:v>
+      </x:c>
+      <x:c r="H26" s="9" t="str">
+        <x:v>functional</x:v>
+      </x:c>
+      <x:c r="I26" s="9" t="str">
+        <x:v>ready</x:v>
+      </x:c>
+      <x:c r="J26" s="9" t="str"/>
+      <x:c r="K26" s="9" t="str">
+        <x:v>outputs/a2-migration-01a0e663/supplier-20260928.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="72" customHeight="1">
+      <x:c r="A27" s="9" t="str">
+        <x:v>SUP-22</x:v>
+      </x:c>
+      <x:c r="B27" s="9" t="str">
+        <x:v>A2-612640976aeb</x:v>
+      </x:c>
+      <x:c r="C27" s="9" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D27" s="9" t="str">
+        <x:v>Multiple delete/reload</x:v>
+      </x:c>
+      <x:c r="E27" s="9" t="str">
+        <x:v>Own A/B/C supplier fixtures; reportdagi data aliaslar</x:v>
+      </x:c>
+      <x:c r="F27" s="9" t="str">
+        <x:v>A ni qayta qo‘shish; A/B → Удалить 2 → Да; reload</x:v>
+      </x:c>
+      <x:c r="G27" s="9" t="str">
+        <x:v>Ikkala supplier yo‘q, empty-state barqaror</x:v>
+      </x:c>
+      <x:c r="H27" s="9" t="str">
+        <x:v>functional</x:v>
+      </x:c>
+      <x:c r="I27" s="9" t="str">
+        <x:v>ready</x:v>
+      </x:c>
+      <x:c r="J27" s="9" t="str"/>
+      <x:c r="K27" s="9" t="str">
+        <x:v>outputs/a2-migration-01a0e663/supplier-20260928.md</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:dataValidations count="2">
@@ -44604,7 +45392,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R183cf548e3834286"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1d046da170c74bd2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -44665,7 +45453,7 @@
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
       <x:c r="A3" s="4" t="str">
-        <x:v>Har bir urinish alohida yoziladi. Retest eski natijani almashtirmaydi.</x:v>
+        <x:v>Manual UI tekshiruv. Sana — sessiya sanasi; aniq amal vaqtlari o‘lchanmagan. Avtotest run qilinmagan.</x:v>
       </x:c>
       <x:c r="B3" s="2"/>
       <x:c r="C3" s="2"/>
@@ -44741,90 +45529,973 @@
         <x:v>Bajaruvchi</x:v>
       </x:c>
     </x:row>
-    <x:row r="6" ht="24" customHeight="1">
-      <x:c r="A6" s="2"/>
-      <x:c r="B6" s="2"/>
-      <x:c r="C6" s="2"/>
-      <x:c r="D6" s="2"/>
-      <x:c r="E6" s="12"/>
-      <x:c r="F6" s="2"/>
-      <x:c r="G6" s="2"/>
-      <x:c r="H6" s="2"/>
-      <x:c r="I6" s="2"/>
-      <x:c r="J6" s="2"/>
-      <x:c r="K6" s="2"/>
-      <x:c r="L6" s="2"/>
-      <x:c r="M6" s="2"/>
-      <x:c r="N6" s="2"/>
-    </x:row>
-    <x:row r="7">
-      <x:c r="E7" s="13"/>
-    </x:row>
-    <x:row r="8">
-      <x:c r="E8" s="13"/>
-    </x:row>
-    <x:row r="9">
-      <x:c r="E9" s="13"/>
-    </x:row>
-    <x:row r="10">
-      <x:c r="E10" s="13"/>
-    </x:row>
-    <x:row r="11">
-      <x:c r="E11" s="13"/>
-    </x:row>
-    <x:row r="12">
-      <x:c r="E12" s="13"/>
-    </x:row>
-    <x:row r="13">
-      <x:c r="E13" s="13"/>
-    </x:row>
-    <x:row r="14">
-      <x:c r="E14" s="13"/>
-    </x:row>
-    <x:row r="15">
-      <x:c r="E15" s="13"/>
-    </x:row>
-    <x:row r="16">
-      <x:c r="E16" s="13"/>
-    </x:row>
-    <x:row r="17">
-      <x:c r="E17" s="13"/>
-    </x:row>
-    <x:row r="18">
-      <x:c r="E18" s="13"/>
-    </x:row>
-    <x:row r="19">
-      <x:c r="E19" s="13"/>
-    </x:row>
-    <x:row r="20">
-      <x:c r="E20" s="13"/>
-    </x:row>
-    <x:row r="21">
-      <x:c r="E21" s="13"/>
-    </x:row>
-    <x:row r="22">
-      <x:c r="E22" s="13"/>
-    </x:row>
-    <x:row r="23">
-      <x:c r="E23" s="13"/>
-    </x:row>
-    <x:row r="24">
-      <x:c r="E24" s="13"/>
-    </x:row>
-    <x:row r="25">
-      <x:c r="E25" s="13"/>
-    </x:row>
-    <x:row r="26">
-      <x:c r="E26" s="13"/>
-    </x:row>
-    <x:row r="27">
-      <x:c r="E27" s="13"/>
-    </x:row>
-    <x:row r="28">
-      <x:c r="E28" s="13"/>
-    </x:row>
-    <x:row r="29">
-      <x:c r="E29" s="13"/>
+    <x:row r="6" ht="72" customHeight="1">
+      <x:c r="A6" s="9" t="str">
+        <x:v>SUP-R01</x:v>
+      </x:c>
+      <x:c r="B6" s="9" t="str">
+        <x:v>SUP-01</x:v>
+      </x:c>
+      <x:c r="C6" s="9" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D6" s="9" t="str">
+        <x:v>A2-c6398bcf3bba</x:v>
+      </x:c>
+      <x:c r="E6" s="21" t="str">
+        <x:v>2026-09-28</x:v>
+      </x:c>
+      <x:c r="F6" s="9" t="str">
+        <x:v>Xtrade A2; build unknown</x:v>
+      </x:c>
+      <x:c r="G6" s="9" t="str">
+        <x:v>Admin / filial-pw157168 / A,B,C</x:v>
+      </x:c>
+      <x:c r="H6" s="9" t="str">
+        <x:v>manual</x:v>
+      </x:c>
+      <x:c r="I6" s="9" t="str">
+        <x:v>passed</x:v>
+      </x:c>
+      <x:c r="J6" s="9" t="str">
+        <x:v>Status/type/Name/VAT/VAT%/Excise aniqlandi; bo‘sh Save disabled.</x:v>
+      </x:c>
+      <x:c r="K6" s="9" t="str">
+        <x:v>outputs/a2-migration-01a0e663/supplier-20260928.md</x:v>
+      </x:c>
+      <x:c r="L6" s="9" t="str"/>
+      <x:c r="M6" s="9" t="str"/>
+      <x:c r="N6" s="9" t="str">
+        <x:v>Codex UI session</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="72" customHeight="1">
+      <x:c r="A7" s="9" t="str">
+        <x:v>SUP-R02</x:v>
+      </x:c>
+      <x:c r="B7" s="9" t="str">
+        <x:v>SUP-02</x:v>
+      </x:c>
+      <x:c r="C7" s="9" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D7" s="9" t="str">
+        <x:v>A2-c6398bcf3bba</x:v>
+      </x:c>
+      <x:c r="E7" s="21" t="str">
+        <x:v>2026-09-28</x:v>
+      </x:c>
+      <x:c r="F7" s="9" t="str">
+        <x:v>Xtrade A2; build unknown</x:v>
+      </x:c>
+      <x:c r="G7" s="9" t="str">
+        <x:v>Admin / filial-pw157168 / A,B,C</x:v>
+      </x:c>
+      <x:c r="H7" s="9" t="str">
+        <x:v>manual</x:v>
+      </x:c>
+      <x:c r="I7" s="9" t="str">
+        <x:v>passed</x:v>
+      </x:c>
+      <x:c r="J7" s="9" t="str">
+        <x:v>A va B legal supplier listda paydo bo‘ldi.</x:v>
+      </x:c>
+      <x:c r="K7" s="9" t="str">
+        <x:v>outputs/a2-migration-01a0e663/supplier-20260928.md</x:v>
+      </x:c>
+      <x:c r="L7" s="9" t="str"/>
+      <x:c r="M7" s="9" t="str"/>
+      <x:c r="N7" s="9" t="str">
+        <x:v>Codex UI session</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="72" customHeight="1">
+      <x:c r="A8" s="9" t="str">
+        <x:v>SUP-R03a</x:v>
+      </x:c>
+      <x:c r="B8" s="9" t="str">
+        <x:v>SUP-03</x:v>
+      </x:c>
+      <x:c r="C8" s="9" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D8" s="9" t="str">
+        <x:v>A2-c6398bcf3bba</x:v>
+      </x:c>
+      <x:c r="E8" s="21" t="str">
+        <x:v>2026-09-28</x:v>
+      </x:c>
+      <x:c r="F8" s="9" t="str">
+        <x:v>Xtrade A2; build unknown</x:v>
+      </x:c>
+      <x:c r="G8" s="9" t="str">
+        <x:v>Admin / filial-pw157168 / A,B,C</x:v>
+      </x:c>
+      <x:c r="H8" s="9" t="str">
+        <x:v>manual</x:v>
+      </x:c>
+      <x:c r="I8" s="9" t="str">
+        <x:v>needs_review</x:v>
+      </x:c>
+      <x:c r="J8" s="9" t="str">
+        <x:v>Name fill + Save natija bermadi. App bug tasdiqlanmagan; autocomplete commit tekshirildi.</x:v>
+      </x:c>
+      <x:c r="K8" s="9" t="str">
+        <x:v>outputs/a2-migration-01a0e663/supplier-20260928.md</x:v>
+      </x:c>
+      <x:c r="L8" s="9" t="str"/>
+      <x:c r="M8" s="9" t="str"/>
+      <x:c r="N8" s="9" t="str">
+        <x:v>Codex UI session</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="72" customHeight="1">
+      <x:c r="A9" s="9" t="str">
+        <x:v>SUP-R03</x:v>
+      </x:c>
+      <x:c r="B9" s="9" t="str">
+        <x:v>SUP-03</x:v>
+      </x:c>
+      <x:c r="C9" s="9" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D9" s="9" t="str">
+        <x:v>A2-c6398bcf3bba</x:v>
+      </x:c>
+      <x:c r="E9" s="21" t="str">
+        <x:v>2026-09-28</x:v>
+      </x:c>
+      <x:c r="F9" s="9" t="str">
+        <x:v>Xtrade A2; build unknown</x:v>
+      </x:c>
+      <x:c r="G9" s="9" t="str">
+        <x:v>Admin / filial-pw157168 / A,B,C</x:v>
+      </x:c>
+      <x:c r="H9" s="9" t="str">
+        <x:v>manual</x:v>
+      </x:c>
+      <x:c r="I9" s="9" t="str">
+        <x:v>passed</x:v>
+      </x:c>
+      <x:c r="J9" s="9" t="str">
+        <x:v>C yaratildi; code/name/natural/active mos. Dastlabki urinish alohida qaydda.</x:v>
+      </x:c>
+      <x:c r="K9" s="9" t="str">
+        <x:v>outputs/a2-migration-01a0e663/supplier-20260928.md</x:v>
+      </x:c>
+      <x:c r="L9" s="9" t="str"/>
+      <x:c r="M9" s="9" t="str">
+        <x:v>SUP-R03a</x:v>
+      </x:c>
+      <x:c r="N9" s="9" t="str">
+        <x:v>Codex UI session</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="72" customHeight="1">
+      <x:c r="A10" s="9" t="str">
+        <x:v>SUP-R04</x:v>
+      </x:c>
+      <x:c r="B10" s="9" t="str">
+        <x:v>SUP-04</x:v>
+      </x:c>
+      <x:c r="C10" s="9" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D10" s="9" t="str">
+        <x:v>A2-358b793d482a</x:v>
+      </x:c>
+      <x:c r="E10" s="21" t="str">
+        <x:v>2026-09-28</x:v>
+      </x:c>
+      <x:c r="F10" s="9" t="str">
+        <x:v>Xtrade A2; build unknown</x:v>
+      </x:c>
+      <x:c r="G10" s="9" t="str">
+        <x:v>Admin / filial-pw157168 / A,B,C</x:v>
+      </x:c>
+      <x:c r="H10" s="9" t="str">
+        <x:v>manual</x:v>
+      </x:c>
+      <x:c r="I10" s="9" t="str">
+        <x:v>passed</x:v>
+      </x:c>
+      <x:c r="J10" s="9" t="str">
+        <x:v>A legal/VAT12/active, C natural/active va code/name to‘g‘ri.</x:v>
+      </x:c>
+      <x:c r="K10" s="9" t="str">
+        <x:v>outputs/a2-migration-01a0e663/supplier-20260928.md</x:v>
+      </x:c>
+      <x:c r="L10" s="9" t="str"/>
+      <x:c r="M10" s="9" t="str"/>
+      <x:c r="N10" s="9" t="str">
+        <x:v>Codex UI session</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="72" customHeight="1">
+      <x:c r="A11" s="9" t="str">
+        <x:v>SUP-R05</x:v>
+      </x:c>
+      <x:c r="B11" s="9" t="str">
+        <x:v>SUP-05</x:v>
+      </x:c>
+      <x:c r="C11" s="9" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D11" s="9" t="str">
+        <x:v>A2-358b793d482a</x:v>
+      </x:c>
+      <x:c r="E11" s="21" t="str">
+        <x:v>2026-09-28</x:v>
+      </x:c>
+      <x:c r="F11" s="9" t="str">
+        <x:v>Xtrade A2; build unknown</x:v>
+      </x:c>
+      <x:c r="G11" s="9" t="str">
+        <x:v>Admin / filial-pw157168 / A,B,C</x:v>
+      </x:c>
+      <x:c r="H11" s="9" t="str">
+        <x:v>manual</x:v>
+      </x:c>
+      <x:c r="I11" s="9" t="str">
+        <x:v>passed</x:v>
+      </x:c>
+      <x:c r="J11" s="9" t="str">
+        <x:v>Xatosiz ochildi; historyda A create/VAT12 bor. Hujjatli tablar empty-state bilan tekshirildi.</x:v>
+      </x:c>
+      <x:c r="K11" s="9" t="str">
+        <x:v>outputs/a2-migration-01a0e663/supplier-20260928.md</x:v>
+      </x:c>
+      <x:c r="L11" s="9" t="str"/>
+      <x:c r="M11" s="9" t="str"/>
+      <x:c r="N11" s="9" t="str">
+        <x:v>Codex UI session</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="72" customHeight="1">
+      <x:c r="A12" s="9" t="str">
+        <x:v>SUP-R06</x:v>
+      </x:c>
+      <x:c r="B12" s="9" t="str">
+        <x:v>SUP-06</x:v>
+      </x:c>
+      <x:c r="C12" s="9" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D12" s="9" t="str">
+        <x:v>A2-358b793d482a</x:v>
+      </x:c>
+      <x:c r="E12" s="21" t="str">
+        <x:v>2026-09-28</x:v>
+      </x:c>
+      <x:c r="F12" s="9" t="str">
+        <x:v>Xtrade A2; build unknown</x:v>
+      </x:c>
+      <x:c r="G12" s="9" t="str">
+        <x:v>Admin / filial-pw157168 / A,B,C</x:v>
+      </x:c>
+      <x:c r="H12" s="9" t="str">
+        <x:v>manual</x:v>
+      </x:c>
+      <x:c r="I12" s="9" t="str">
+        <x:v>failed</x:v>
+      </x:c>
+      <x:c r="J12" s="9" t="str">
+        <x:v>Ошибка: URL: anor/mkw/supplier_view:purchase. A va C da takrorlandi.</x:v>
+      </x:c>
+      <x:c r="K12" s="9" t="str">
+        <x:v>outputs/a2-migration-01a0e663/supplier-20260928.md</x:v>
+      </x:c>
+      <x:c r="L12" s="9" t="str">
+        <x:v>SUP-001</x:v>
+      </x:c>
+      <x:c r="M12" s="9" t="str"/>
+      <x:c r="N12" s="9" t="str">
+        <x:v>Codex UI session</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="72" customHeight="1">
+      <x:c r="A13" s="9" t="str">
+        <x:v>SUP-R07</x:v>
+      </x:c>
+      <x:c r="B13" s="9" t="str">
+        <x:v>SUP-07</x:v>
+      </x:c>
+      <x:c r="C13" s="9" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D13" s="9" t="str">
+        <x:v>A2-84e0eb5cd0a4</x:v>
+      </x:c>
+      <x:c r="E13" s="21" t="str">
+        <x:v>2026-09-28</x:v>
+      </x:c>
+      <x:c r="F13" s="9" t="str">
+        <x:v>Xtrade A2; build unknown</x:v>
+      </x:c>
+      <x:c r="G13" s="9" t="str">
+        <x:v>Admin / filial-pw157168 / A,B,C</x:v>
+      </x:c>
+      <x:c r="H13" s="9" t="str">
+        <x:v>manual</x:v>
+      </x:c>
+      <x:c r="I13" s="9" t="str">
+        <x:v>passed</x:v>
+      </x:c>
+      <x:c r="J13" s="9" t="str">
+        <x:v>VAT15, inactive, excise false saqlandi. Type/name readonly. Listdan edit ham ochildi.</x:v>
+      </x:c>
+      <x:c r="K13" s="9" t="str">
+        <x:v>outputs/a2-migration-01a0e663/supplier-20260928.md</x:v>
+      </x:c>
+      <x:c r="L13" s="9" t="str"/>
+      <x:c r="M13" s="9" t="str"/>
+      <x:c r="N13" s="9" t="str">
+        <x:v>Codex UI session</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="72" customHeight="1">
+      <x:c r="A14" s="9" t="str">
+        <x:v>SUP-R08</x:v>
+      </x:c>
+      <x:c r="B14" s="9" t="str">
+        <x:v>SUP-08</x:v>
+      </x:c>
+      <x:c r="C14" s="9" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D14" s="9" t="str">
+        <x:v>A2-612640976aeb</x:v>
+      </x:c>
+      <x:c r="E14" s="21" t="str">
+        <x:v>2026-09-28</x:v>
+      </x:c>
+      <x:c r="F14" s="9" t="str">
+        <x:v>Xtrade A2; build unknown</x:v>
+      </x:c>
+      <x:c r="G14" s="9" t="str">
+        <x:v>Admin / filial-pw157168 / A,B,C</x:v>
+      </x:c>
+      <x:c r="H14" s="9" t="str">
+        <x:v>manual</x:v>
+      </x:c>
+      <x:c r="I14" s="9" t="str">
+        <x:v>passed</x:v>
+      </x:c>
+      <x:c r="J14" s="9" t="str">
+        <x:v>A active, C inactive row matni tekshirildi.</x:v>
+      </x:c>
+      <x:c r="K14" s="9" t="str">
+        <x:v>outputs/a2-migration-01a0e663/supplier-20260928.md</x:v>
+      </x:c>
+      <x:c r="L14" s="9" t="str"/>
+      <x:c r="M14" s="9" t="str"/>
+      <x:c r="N14" s="9" t="str">
+        <x:v>Codex UI session</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="72" customHeight="1">
+      <x:c r="A15" s="9" t="str">
+        <x:v>SUP-R09</x:v>
+      </x:c>
+      <x:c r="B15" s="9" t="str">
+        <x:v>SUP-09</x:v>
+      </x:c>
+      <x:c r="C15" s="9" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D15" s="9" t="str">
+        <x:v>A2-c286a891c1bf</x:v>
+      </x:c>
+      <x:c r="E15" s="21" t="str">
+        <x:v>2026-09-28</x:v>
+      </x:c>
+      <x:c r="F15" s="9" t="str">
+        <x:v>Xtrade A2; build unknown</x:v>
+      </x:c>
+      <x:c r="G15" s="9" t="str">
+        <x:v>Admin / filial-pw157168 / A,B,C</x:v>
+      </x:c>
+      <x:c r="H15" s="9" t="str">
+        <x:v>manual</x:v>
+      </x:c>
+      <x:c r="I15" s="9" t="str">
+        <x:v>passed</x:v>
+      </x:c>
+      <x:c r="J15" s="9" t="str">
+        <x:v>Attached: product-pw157168, 1/1.</x:v>
+      </x:c>
+      <x:c r="K15" s="9" t="str">
+        <x:v>outputs/a2-migration-01a0e663/supplier-20260928.md</x:v>
+      </x:c>
+      <x:c r="L15" s="9" t="str"/>
+      <x:c r="M15" s="9" t="str"/>
+      <x:c r="N15" s="9" t="str">
+        <x:v>Codex UI session</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="72" customHeight="1">
+      <x:c r="A16" s="9" t="str">
+        <x:v>SUP-R10</x:v>
+      </x:c>
+      <x:c r="B16" s="9" t="str">
+        <x:v>SUP-10</x:v>
+      </x:c>
+      <x:c r="C16" s="9" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D16" s="9" t="str">
+        <x:v>A2-c286a891c1bf</x:v>
+      </x:c>
+      <x:c r="E16" s="21" t="str">
+        <x:v>2026-09-28</x:v>
+      </x:c>
+      <x:c r="F16" s="9" t="str">
+        <x:v>Xtrade A2; build unknown</x:v>
+      </x:c>
+      <x:c r="G16" s="9" t="str">
+        <x:v>Admin / filial-pw157168 / A,B,C</x:v>
+      </x:c>
+      <x:c r="H16" s="9" t="str">
+        <x:v>manual</x:v>
+      </x:c>
+      <x:c r="I16" s="9" t="str">
+        <x:v>passed</x:v>
+      </x:c>
+      <x:c r="J16" s="9" t="str">
+        <x:v>Attached empty; product Availableda qaytdi.</x:v>
+      </x:c>
+      <x:c r="K16" s="9" t="str">
+        <x:v>outputs/a2-migration-01a0e663/supplier-20260928.md</x:v>
+      </x:c>
+      <x:c r="L16" s="9" t="str"/>
+      <x:c r="M16" s="9" t="str"/>
+      <x:c r="N16" s="9" t="str">
+        <x:v>Codex UI session</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="72" customHeight="1">
+      <x:c r="A17" s="9" t="str">
+        <x:v>SUP-R11</x:v>
+      </x:c>
+      <x:c r="B17" s="9" t="str">
+        <x:v>SUP-11</x:v>
+      </x:c>
+      <x:c r="C17" s="9" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D17" s="9" t="str">
+        <x:v>A2-c286a891c1bf</x:v>
+      </x:c>
+      <x:c r="E17" s="21" t="str">
+        <x:v>2026-09-28</x:v>
+      </x:c>
+      <x:c r="F17" s="9" t="str">
+        <x:v>Xtrade A2; build unknown</x:v>
+      </x:c>
+      <x:c r="G17" s="9" t="str">
+        <x:v>Admin / filial-pw157168 / A,B,C</x:v>
+      </x:c>
+      <x:c r="H17" s="9" t="str">
+        <x:v>manual</x:v>
+      </x:c>
+      <x:c r="I17" s="9" t="str">
+        <x:v>passed</x:v>
+      </x:c>
+      <x:c r="J17" s="9" t="str">
+        <x:v>Ikkala product kodi Attached ro‘yxatda.</x:v>
+      </x:c>
+      <x:c r="K17" s="9" t="str">
+        <x:v>outputs/a2-migration-01a0e663/supplier-20260928.md</x:v>
+      </x:c>
+      <x:c r="L17" s="9" t="str"/>
+      <x:c r="M17" s="9" t="str"/>
+      <x:c r="N17" s="9" t="str">
+        <x:v>Codex UI session</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="72" customHeight="1">
+      <x:c r="A18" s="9" t="str">
+        <x:v>SUP-R12</x:v>
+      </x:c>
+      <x:c r="B18" s="9" t="str">
+        <x:v>SUP-12</x:v>
+      </x:c>
+      <x:c r="C18" s="9" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D18" s="9" t="str">
+        <x:v>A2-c286a891c1bf</x:v>
+      </x:c>
+      <x:c r="E18" s="21" t="str">
+        <x:v>2026-09-28</x:v>
+      </x:c>
+      <x:c r="F18" s="9" t="str">
+        <x:v>Xtrade A2; build unknown</x:v>
+      </x:c>
+      <x:c r="G18" s="9" t="str">
+        <x:v>Admin / filial-pw157168 / A,B,C</x:v>
+      </x:c>
+      <x:c r="H18" s="9" t="str">
+        <x:v>manual</x:v>
+      </x:c>
+      <x:c r="I18" s="9" t="str">
+        <x:v>passed</x:v>
+      </x:c>
+      <x:c r="J18" s="9" t="str">
+        <x:v>Attached: 0/0.</x:v>
+      </x:c>
+      <x:c r="K18" s="9" t="str">
+        <x:v>outputs/a2-migration-01a0e663/supplier-20260928.md</x:v>
+      </x:c>
+      <x:c r="L18" s="9" t="str"/>
+      <x:c r="M18" s="9" t="str"/>
+      <x:c r="N18" s="9" t="str">
+        <x:v>Codex UI session</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="72" customHeight="1">
+      <x:c r="A19" s="9" t="str">
+        <x:v>SUP-R13</x:v>
+      </x:c>
+      <x:c r="B19" s="9" t="str">
+        <x:v>SUP-13</x:v>
+      </x:c>
+      <x:c r="C19" s="9" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D19" s="9" t="str">
+        <x:v>A2-612640976aeb</x:v>
+      </x:c>
+      <x:c r="E19" s="21" t="str">
+        <x:v>2026-09-28</x:v>
+      </x:c>
+      <x:c r="F19" s="9" t="str">
+        <x:v>Xtrade A2; build unknown</x:v>
+      </x:c>
+      <x:c r="G19" s="9" t="str">
+        <x:v>Admin / filial-pw157168 / A,B,C</x:v>
+      </x:c>
+      <x:c r="H19" s="9" t="str">
+        <x:v>manual</x:v>
+      </x:c>
+      <x:c r="I19" s="9" t="str">
+        <x:v>passed</x:v>
+      </x:c>
+      <x:c r="J19" s="9" t="str">
+        <x:v>B mavjud, A yo‘q, 1/1.</x:v>
+      </x:c>
+      <x:c r="K19" s="9" t="str">
+        <x:v>outputs/a2-migration-01a0e663/supplier-20260928.md</x:v>
+      </x:c>
+      <x:c r="L19" s="9" t="str"/>
+      <x:c r="M19" s="9" t="str"/>
+      <x:c r="N19" s="9" t="str">
+        <x:v>Codex UI session</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="72" customHeight="1">
+      <x:c r="A20" s="9" t="str">
+        <x:v>SUP-R14</x:v>
+      </x:c>
+      <x:c r="B20" s="9" t="str">
+        <x:v>SUP-14</x:v>
+      </x:c>
+      <x:c r="C20" s="9" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D20" s="9" t="str">
+        <x:v>A2-612640976aeb</x:v>
+      </x:c>
+      <x:c r="E20" s="21" t="str">
+        <x:v>2026-09-28</x:v>
+      </x:c>
+      <x:c r="F20" s="9" t="str">
+        <x:v>Xtrade A2; build unknown</x:v>
+      </x:c>
+      <x:c r="G20" s="9" t="str">
+        <x:v>Admin / filial-pw157168 / A,B,C</x:v>
+      </x:c>
+      <x:c r="H20" s="9" t="str">
+        <x:v>manual</x:v>
+      </x:c>
+      <x:c r="I20" s="9" t="str">
+        <x:v>passed</x:v>
+      </x:c>
+      <x:c r="J20" s="9" t="str">
+        <x:v>0/0 → A/B 2/2. fill-empty no-op test/tool kuzatuvi alohida qayd.</x:v>
+      </x:c>
+      <x:c r="K20" s="9" t="str">
+        <x:v>outputs/a2-migration-01a0e663/supplier-20260928.md</x:v>
+      </x:c>
+      <x:c r="L20" s="9" t="str"/>
+      <x:c r="M20" s="9" t="str"/>
+      <x:c r="N20" s="9" t="str">
+        <x:v>Codex UI session</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="72" customHeight="1">
+      <x:c r="A21" s="9" t="str">
+        <x:v>SUP-R15</x:v>
+      </x:c>
+      <x:c r="B21" s="9" t="str">
+        <x:v>SUP-15</x:v>
+      </x:c>
+      <x:c r="C21" s="9" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D21" s="9" t="str">
+        <x:v>A2-612640976aeb</x:v>
+      </x:c>
+      <x:c r="E21" s="21" t="str">
+        <x:v>2026-09-28</x:v>
+      </x:c>
+      <x:c r="F21" s="9" t="str">
+        <x:v>Xtrade A2; build unknown</x:v>
+      </x:c>
+      <x:c r="G21" s="9" t="str">
+        <x:v>Admin / filial-pw157168 / A,B,C</x:v>
+      </x:c>
+      <x:c r="H21" s="9" t="str">
+        <x:v>manual</x:v>
+      </x:c>
+      <x:c r="I21" s="9" t="str">
+        <x:v>passed</x:v>
+      </x:c>
+      <x:c r="J21" s="9" t="str">
+        <x:v>A bor, B yo‘q.</x:v>
+      </x:c>
+      <x:c r="K21" s="9" t="str">
+        <x:v>outputs/a2-migration-01a0e663/supplier-20260928.md</x:v>
+      </x:c>
+      <x:c r="L21" s="9" t="str"/>
+      <x:c r="M21" s="9" t="str"/>
+      <x:c r="N21" s="9" t="str">
+        <x:v>Codex UI session</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="72" customHeight="1">
+      <x:c r="A22" s="9" t="str">
+        <x:v>SUP-R16</x:v>
+      </x:c>
+      <x:c r="B22" s="9" t="str">
+        <x:v>SUP-16</x:v>
+      </x:c>
+      <x:c r="C22" s="9" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D22" s="9" t="str">
+        <x:v>A2-612640976aeb</x:v>
+      </x:c>
+      <x:c r="E22" s="21" t="str">
+        <x:v>2026-09-28</x:v>
+      </x:c>
+      <x:c r="F22" s="9" t="str">
+        <x:v>Xtrade A2; build unknown</x:v>
+      </x:c>
+      <x:c r="G22" s="9" t="str">
+        <x:v>Admin / filial-pw157168 / A,B,C</x:v>
+      </x:c>
+      <x:c r="H22" s="9" t="str">
+        <x:v>manual</x:v>
+      </x:c>
+      <x:c r="I22" s="9" t="str">
+        <x:v>passed</x:v>
+      </x:c>
+      <x:c r="J22" s="9" t="str">
+        <x:v>Empty → A/B qaytdi.</x:v>
+      </x:c>
+      <x:c r="K22" s="9" t="str">
+        <x:v>outputs/a2-migration-01a0e663/supplier-20260928.md</x:v>
+      </x:c>
+      <x:c r="L22" s="9" t="str"/>
+      <x:c r="M22" s="9" t="str"/>
+      <x:c r="N22" s="9" t="str">
+        <x:v>Codex UI session</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="72" customHeight="1">
+      <x:c r="A23" s="9" t="str">
+        <x:v>SUP-R17</x:v>
+      </x:c>
+      <x:c r="B23" s="9" t="str">
+        <x:v>SUP-17</x:v>
+      </x:c>
+      <x:c r="C23" s="9" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D23" s="9" t="str">
+        <x:v>A2-612640976aeb</x:v>
+      </x:c>
+      <x:c r="E23" s="21" t="str">
+        <x:v>2026-09-28</x:v>
+      </x:c>
+      <x:c r="F23" s="9" t="str">
+        <x:v>Xtrade A2; build unknown</x:v>
+      </x:c>
+      <x:c r="G23" s="9" t="str">
+        <x:v>Admin / filial-pw157168 / A,B,C</x:v>
+      </x:c>
+      <x:c r="H23" s="9" t="str">
+        <x:v>manual</x:v>
+      </x:c>
+      <x:c r="I23" s="9" t="str">
+        <x:v>passed</x:v>
+      </x:c>
+      <x:c r="J23" s="9" t="str">
+        <x:v>A/B inactive; keyin A/B active.</x:v>
+      </x:c>
+      <x:c r="K23" s="9" t="str">
+        <x:v>outputs/a2-migration-01a0e663/supplier-20260928.md</x:v>
+      </x:c>
+      <x:c r="L23" s="9" t="str"/>
+      <x:c r="M23" s="9" t="str"/>
+      <x:c r="N23" s="9" t="str">
+        <x:v>Codex UI session</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="72" customHeight="1">
+      <x:c r="A24" s="9" t="str">
+        <x:v>SUP-R18</x:v>
+      </x:c>
+      <x:c r="B24" s="9" t="str">
+        <x:v>SUP-18</x:v>
+      </x:c>
+      <x:c r="C24" s="9" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D24" s="9" t="str">
+        <x:v>A2-612640976aeb</x:v>
+      </x:c>
+      <x:c r="E24" s="21" t="str">
+        <x:v>2026-09-28</x:v>
+      </x:c>
+      <x:c r="F24" s="9" t="str">
+        <x:v>Xtrade A2; build unknown</x:v>
+      </x:c>
+      <x:c r="G24" s="9" t="str">
+        <x:v>Admin / filial-pw157168 / A,B,C</x:v>
+      </x:c>
+      <x:c r="H24" s="9" t="str">
+        <x:v>manual</x:v>
+      </x:c>
+      <x:c r="I24" s="9" t="str">
+        <x:v>passed</x:v>
+      </x:c>
+      <x:c r="J24" s="9" t="str">
+        <x:v>12 hodisa, Admin va vaqtlar ko‘rindi.</x:v>
+      </x:c>
+      <x:c r="K24" s="9" t="str">
+        <x:v>outputs/a2-migration-01a0e663/supplier-20260928.md</x:v>
+      </x:c>
+      <x:c r="L24" s="9" t="str"/>
+      <x:c r="M24" s="9" t="str"/>
+      <x:c r="N24" s="9" t="str">
+        <x:v>Codex UI session</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="72" customHeight="1">
+      <x:c r="A25" s="9" t="str">
+        <x:v>SUP-R19</x:v>
+      </x:c>
+      <x:c r="B25" s="9" t="str">
+        <x:v>SUP-19</x:v>
+      </x:c>
+      <x:c r="C25" s="9" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D25" s="9" t="str">
+        <x:v>A2-432abf130d2e</x:v>
+      </x:c>
+      <x:c r="E25" s="21" t="str">
+        <x:v>2026-09-28</x:v>
+      </x:c>
+      <x:c r="F25" s="9" t="str">
+        <x:v>Xtrade A2; build unknown</x:v>
+      </x:c>
+      <x:c r="G25" s="9" t="str">
+        <x:v>Admin / filial-pw157168 / A,B,C</x:v>
+      </x:c>
+      <x:c r="H25" s="9" t="str">
+        <x:v>manual</x:v>
+      </x:c>
+      <x:c r="I25" s="9" t="str">
+        <x:v>passed</x:v>
+      </x:c>
+      <x:c r="J25" s="9" t="str">
+        <x:v>4 maydon/qiymat mos.</x:v>
+      </x:c>
+      <x:c r="K25" s="9" t="str">
+        <x:v>outputs/a2-migration-01a0e663/supplier-20260928.md</x:v>
+      </x:c>
+      <x:c r="L25" s="9" t="str"/>
+      <x:c r="M25" s="9" t="str"/>
+      <x:c r="N25" s="9" t="str">
+        <x:v>Codex UI session</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="72" customHeight="1">
+      <x:c r="A26" s="9" t="str">
+        <x:v>SUP-R20</x:v>
+      </x:c>
+      <x:c r="B26" s="9" t="str">
+        <x:v>SUP-20</x:v>
+      </x:c>
+      <x:c r="C26" s="9" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D26" s="9" t="str">
+        <x:v>A2-612640976aeb</x:v>
+      </x:c>
+      <x:c r="E26" s="21" t="str">
+        <x:v>2026-09-28</x:v>
+      </x:c>
+      <x:c r="F26" s="9" t="str">
+        <x:v>Xtrade A2; build unknown</x:v>
+      </x:c>
+      <x:c r="G26" s="9" t="str">
+        <x:v>Admin / filial-pw157168 / A,B,C</x:v>
+      </x:c>
+      <x:c r="H26" s="9" t="str">
+        <x:v>manual</x:v>
+      </x:c>
+      <x:c r="I26" s="9" t="str">
+        <x:v>passed</x:v>
+      </x:c>
+      <x:c r="J26" s="9" t="str">
+        <x:v>A/B listda qoldi.</x:v>
+      </x:c>
+      <x:c r="K26" s="9" t="str">
+        <x:v>outputs/a2-migration-01a0e663/supplier-20260928.md</x:v>
+      </x:c>
+      <x:c r="L26" s="9" t="str"/>
+      <x:c r="M26" s="9" t="str"/>
+      <x:c r="N26" s="9" t="str">
+        <x:v>Codex UI session</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="72" customHeight="1">
+      <x:c r="A27" s="9" t="str">
+        <x:v>SUP-R21</x:v>
+      </x:c>
+      <x:c r="B27" s="9" t="str">
+        <x:v>SUP-21</x:v>
+      </x:c>
+      <x:c r="C27" s="9" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D27" s="9" t="str">
+        <x:v>A2-612640976aeb</x:v>
+      </x:c>
+      <x:c r="E27" s="21" t="str">
+        <x:v>2026-09-28</x:v>
+      </x:c>
+      <x:c r="F27" s="9" t="str">
+        <x:v>Xtrade A2; build unknown</x:v>
+      </x:c>
+      <x:c r="G27" s="9" t="str">
+        <x:v>Admin / filial-pw157168 / A,B,C</x:v>
+      </x:c>
+      <x:c r="H27" s="9" t="str">
+        <x:v>manual</x:v>
+      </x:c>
+      <x:c r="I27" s="9" t="str">
+        <x:v>passed</x:v>
+      </x:c>
+      <x:c r="J27" s="9" t="str">
+        <x:v>A yo‘q, B bor; C yakunda o‘chirildi.</x:v>
+      </x:c>
+      <x:c r="K27" s="9" t="str">
+        <x:v>outputs/a2-migration-01a0e663/supplier-20260928.md</x:v>
+      </x:c>
+      <x:c r="L27" s="9" t="str"/>
+      <x:c r="M27" s="9" t="str"/>
+      <x:c r="N27" s="9" t="str">
+        <x:v>Codex UI session</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="72" customHeight="1">
+      <x:c r="A28" s="9" t="str">
+        <x:v>SUP-R22</x:v>
+      </x:c>
+      <x:c r="B28" s="9" t="str">
+        <x:v>SUP-22</x:v>
+      </x:c>
+      <x:c r="C28" s="9" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D28" s="9" t="str">
+        <x:v>A2-612640976aeb</x:v>
+      </x:c>
+      <x:c r="E28" s="21" t="str">
+        <x:v>2026-09-28</x:v>
+      </x:c>
+      <x:c r="F28" s="9" t="str">
+        <x:v>Xtrade A2; build unknown</x:v>
+      </x:c>
+      <x:c r="G28" s="9" t="str">
+        <x:v>Admin / filial-pw157168 / A,B,C</x:v>
+      </x:c>
+      <x:c r="H28" s="9" t="str">
+        <x:v>manual</x:v>
+      </x:c>
+      <x:c r="I28" s="9" t="str">
+        <x:v>passed</x:v>
+      </x:c>
+      <x:c r="J28" s="9" t="str">
+        <x:v>0/0; reload ham empty. Oxirida C delete bilan list yana empty.</x:v>
+      </x:c>
+      <x:c r="K28" s="9" t="str">
+        <x:v>outputs/a2-migration-01a0e663/supplier-20260928.md</x:v>
+      </x:c>
+      <x:c r="L28" s="9" t="str"/>
+      <x:c r="M28" s="9" t="str"/>
+      <x:c r="N28" s="9" t="str">
+        <x:v>Codex UI session</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="72" customHeight="1">
+      <x:c r="A29" s="9" t="str">
+        <x:v>SUP-R06b</x:v>
+      </x:c>
+      <x:c r="B29" s="9" t="str">
+        <x:v>SUP-06</x:v>
+      </x:c>
+      <x:c r="C29" s="9" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D29" s="9" t="str">
+        <x:v>A2-358b793d482a</x:v>
+      </x:c>
+      <x:c r="E29" s="21" t="str">
+        <x:v>2026-09-28</x:v>
+      </x:c>
+      <x:c r="F29" s="9" t="str">
+        <x:v>Xtrade A2; build unknown</x:v>
+      </x:c>
+      <x:c r="G29" s="9" t="str">
+        <x:v>Admin / filial-pw157168 / A,B,C</x:v>
+      </x:c>
+      <x:c r="H29" s="9" t="str">
+        <x:v>manual</x:v>
+      </x:c>
+      <x:c r="I29" s="9" t="str">
+        <x:v>failed</x:v>
+      </x:c>
+      <x:c r="J29" s="9" t="str">
+        <x:v>Natural supplier C (369344) view → Закупки: xuddi shu error dialog. Ikkinchi mustaqil reproduction.</x:v>
+      </x:c>
+      <x:c r="K29" s="9" t="str">
+        <x:v>outputs/a2-migration-01a0e663/supplier-20260928.md</x:v>
+      </x:c>
+      <x:c r="L29" s="9" t="str">
+        <x:v>SUP-001</x:v>
+      </x:c>
+      <x:c r="M29" s="9" t="str">
+        <x:v>SUP-R06</x:v>
+      </x:c>
+      <x:c r="N29" s="9" t="str">
+        <x:v>Codex UI session</x:v>
+      </x:c>
     </x:row>
     <x:row r="30">
       <x:c r="E30" s="13"/>
@@ -45376,7 +47047,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R825345f0c4ee48e8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R76bfbb69e6434b0b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -45434,7 +47105,7 @@
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
       <x:c r="A3" s="4" t="str">
-        <x:v>Hozircha tekshiruv bajarilmagan. Bosh jadval bo‘shligi muammo yo‘qligini anglatmaydi.</x:v>
+        <x:v>SUP-001 ochiq: supplier purchase tab xatosi ikki supplier turida takrorlandi.</x:v>
       </x:c>
       <x:c r="B3" s="2"/>
       <x:c r="C3" s="2"/>
@@ -45505,20 +47176,46 @@
         <x:v>Izoh</x:v>
       </x:c>
     </x:row>
-    <x:row r="6" ht="24" customHeight="1">
-      <x:c r="A6" s="2"/>
-      <x:c r="B6" s="2"/>
-      <x:c r="C6" s="2"/>
-      <x:c r="D6" s="2"/>
-      <x:c r="E6" s="2"/>
-      <x:c r="F6" s="2"/>
-      <x:c r="G6" s="2"/>
-      <x:c r="H6" s="2"/>
-      <x:c r="I6" s="2"/>
-      <x:c r="J6" s="2"/>
-      <x:c r="K6" s="2"/>
-      <x:c r="L6" s="2"/>
-      <x:c r="M6" s="2"/>
+    <x:row r="6" ht="72" customHeight="1">
+      <x:c r="A6" s="9" t="str">
+        <x:v>SUP-001</x:v>
+      </x:c>
+      <x:c r="B6" s="9" t="str">
+        <x:v>A2-358b793d482a</x:v>
+      </x:c>
+      <x:c r="C6" s="9" t="str">
+        <x:v>SUP-R06</x:v>
+      </x:c>
+      <x:c r="D6" s="9" t="str">
+        <x:v>Supplier view Закупки tabida error dialog</x:v>
+      </x:c>
+      <x:c r="E6" s="9" t="str">
+        <x:v>app_bug</x:v>
+      </x:c>
+      <x:c r="F6" s="9" t="str">
+        <x:v>medium</x:v>
+      </x:c>
+      <x:c r="G6" s="9" t="str">
+        <x:v>A yoki C supplier → Просмотреть → Закупки</x:v>
+      </x:c>
+      <x:c r="H6" s="9" t="str">
+        <x:v>Xatosiz grid yoki empty-state</x:v>
+      </x:c>
+      <x:c r="I6" s="9" t="str">
+        <x:v>Ошибка: URL: anor/mkw/supplier_view:purchase</x:v>
+      </x:c>
+      <x:c r="J6" s="9" t="str">
+        <x:v>outputs/a2-migration-01a0e663/supplier-20260928.md</x:v>
+      </x:c>
+      <x:c r="K6" s="9" t="str">
+        <x:v>open</x:v>
+      </x:c>
+      <x:c r="L6" s="9" t="str">
+        <x:v>SUP-R06b</x:v>
+      </x:c>
+      <x:c r="M6" s="9" t="str">
+        <x:v>Legal va natural supplierda takrorlandi. HTTP status/root cause aniqlanmagan.</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:conditionalFormatting sqref="K6:K205">
@@ -45539,7 +47236,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4173cd95874641bc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4a435dc1ba104588"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -46287,7 +47984,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc6385e9766c847fe"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R84abb8745cb14ad7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>